<commit_message>
feat(portfolio): publish and link standalone gumroad products (pos fraud, ccm toolkit, gias 2024 matrix)
</commit_message>
<xml_diff>
--- a/public/downloads/Internal_Audit_Report_Evaluation_Matrix_GIAS_2024.xlsx
+++ b/public/downloads/Internal_Audit_Report_Evaluation_Matrix_GIAS_2024.xlsx
@@ -57,7 +57,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -183,6 +183,31 @@
       <name val="Calibri"/>
       <color rgb="FF0F4C81"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="9.5"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="24">
@@ -447,7 +472,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -809,6 +834,10 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1381,7 +1410,7 @@
     <row r="3" ht="36" customHeight="1" s="79">
       <c r="B3" s="127" t="inlineStr">
         <is>
-          <t>Scored from the Global Internal Audit Standards (GIAS 2024 edition, effective 9 January 2025). Prepared by Majid Mumtaz (CIA, ACA, FCCA) | Director, Veritux Advisory | Author of The Audit Signal. Professional QAIP gate and engagement scoring architecture.</t>
+          <t>Scored from the Global Internal Audit Standards (GIAS 2024 edition, effective 9 January 2025). Prepared by Majid Mumtaz | CIA, ACA, FCCA, GRCP, GRCA, COSO ERM | Director of Internal Audit &amp; Risk Advisory, Veritux Advisory | Author of The Audit Signal. Professional QAIP gate and engagement scoring architecture.</t>
         </is>
       </c>
     </row>
@@ -1723,21 +1752,21 @@
     <row r="40" ht="48" customHeight="1" s="79">
       <c r="B40" s="128" t="inlineStr">
         <is>
-          <t>Tool: Internal Audit Report Evaluation Matrix (GIAS 2024 Conformance) | Author: Majid Mumtaz (CIA, ACA, FCCA) | Director, Veritux Advisory | Author of The Audit Signal</t>
+          <t>Tool: Internal Audit Report Evaluation Matrix (GIAS 2024 Conformance) | Author: Majid Mumtaz | CIA, ACA, FCCA, GRCP, GRCA, COSO ERM | Director, Veritux Advisory | Author of The Audit Signal</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1" s="79">
       <c r="B41" s="129" t="inlineStr">
         <is>
-          <t>Author &amp; Advisory: Majid Mumtaz (CIA, ACA, FCCA) | Director of Internal Audit &amp; Risk Advisory, Veritux Advisory | Author of The Audit Signal (LinkedIn Newsletter)</t>
+          <t>Author &amp; Advisory: Majid Mumtaz | CIA, ACA, FCCA, GRCP, GRCA, COSO ERM | Director of Internal Audit &amp; Risk Advisory, Veritux Advisory | Author of The Audit Signal (LinkedIn Newsletter)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1" s="79">
       <c r="B42" s="130" t="inlineStr">
         <is>
-          <t>Executive Portfolio: https://majidrajpar.github.io/portfolio_my/  |  Newsletter: https://www.linkedin.com/newsletters/7339153291630510080/  |  LinkedIn: https://www.linkedin.com/in/majid-m-4b097118/</t>
+          <t>Executive Portfolio: https://majidrajpar.github.io/portfolio_my/  |  The Audit Signal Newsletter: https://www.linkedin.com/newsletters/the-audit-signal-7339153291630510080/  |  LinkedIn: https://www.linkedin.com/in/majid-m-4b097118/</t>
         </is>
       </c>
     </row>
@@ -8075,7 +8104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:G44"/>
+  <dimension ref="B2:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="3" customWidth="1" style="79" min="1" max="1"/>
@@ -8774,6 +8803,61 @@
       <c r="E44" s="105" t="n"/>
       <c r="F44" s="105" t="n"/>
       <c r="G44" s="106" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="131" t="inlineStr">
+        <is>
+          <t>FRAMEWORK ARCHITECTURE, QAIP GOVERNANCE &amp; THOUGHT LEADERSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="132" t="inlineStr">
+        <is>
+          <t>Framework Architect:</t>
+        </is>
+      </c>
+      <c r="C46" s="133" t="inlineStr">
+        <is>
+          <t>Majid Mumtaz | CIA (IIA), ACA (ICAEW UK), FCCA (ACCA UK), GRCP &amp; GRCA (OCEG), COSO ERM Certified</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="132" t="inlineStr">
+        <is>
+          <t>The Audit Signal Newsletter:</t>
+        </is>
+      </c>
+      <c r="C47" s="134" t="inlineStr">
+        <is>
+          <t>The Audit Signal — Technical Articles on Continuous Auditing &amp; GIAS 2024 Governance (LinkedIn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="132" t="inlineStr">
+        <is>
+          <t>Continuous Controls Monitoring:</t>
+        </is>
+      </c>
+      <c r="C48" s="134" t="inlineStr">
+        <is>
+          <t>Interactive Audit Portfolio &amp; Tools (majidrajpar.github.io/portfolio_my)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="132" t="inlineStr">
+        <is>
+          <t>Author Executive Profile:</t>
+        </is>
+      </c>
+      <c r="C49" s="134" t="inlineStr">
+        <is>
+          <t>LinkedIn Executive Profile: Majid Mumtaz</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="0" insertColumns="0" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
@@ -8840,6 +8924,11 @@
       <formula>OR(F28=1,F28="1")</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId3"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.5" header="0.25" footer="0.25"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="2"/>

</xml_diff>